<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-09 Le pinceau jaune de Victorina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-09.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-09.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le soleil sur la buée</t>
+          <t>Le pinceau jaune de Victorina</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine, atelier peinture, puis maison</t>
+          <t>école, atelier peinture, puis maison</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>La casserole frémit. La buée fait un rond sur la vitre. Victorina peint un soleil jaune. Un chuchotement lui serre le ventre. Le soir, elle raconte, et le soleil va sur la fenêtre.</t>
+          <t>Le préau sent la laine mouillée. Sur le pinceau jaune, un éclat de pinceau brille. Victorina veut peindre les manteaux, maintenant. Elle plonge trop vite : le jaune court. Elle veut parler maintenant : les mots se perdent. Elle refuse de foncer, attend le silence, raconte. Merci vécu. Sur le jaune, l'éclat de pinceau tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La casserole frémit sur le feu. Une buée ronde s'étale sur la vitre. Ça sent l'orange pelée, un peu vive. Les gouttes d'huile brillent sur les doigts de maman. Papa essuie la table avec une éponge jaune. L'éponge est froide, encore mouillée. Dehors, le village est gris et calme. Victorina, tu vois le rond sur la vitre ? Oui, papa. On dirait un soleil. Maman, je veux un vrai soleil, en jaune. Pour la fenêtre de la cuisine. On pourra le peindre à l'école. Tu écoutes la maîtresse, d'accord ? Oui, maman. Papa glisse un biscuit dans la poche. Le biscuit sent le beurre. Il est pour plus tard. En ce moment, Victorina pousse la porte de l'atelier. La table a une nappe bleue, un peu tâchée. Les pots de peinture sont ouverts. Ça sent le papier mouillé. Un pinceau attend près de l'eau. On écoute d'abord. Ensuite, on peint un rond. Puis on lave les pinceaux. Victorina aime écouter. Elle prend le pinceau. Le bois est lisse, un peu collant. Elle plonge le poil dans le jaune. Le jaune est épais. C'est mon soleil, maîtresse. Oui, Victorina. Tu as bien écouté. Maintenant, on lave les pinceaux. Victorina va vers le bac. L'eau devient un peu jaune. Elle lave le poil, tout doucement. Le soleil reste sur la feuille, encore humide. Près du bac, quelqu'un parle tout bas. Victorina entend parler d'un secret. Son ventre se serre. Ses joues deviennent chaudes. Elle pose le pinceau propre. Je raconterai à la maison. Le soir, la casserole frémit encore. La buée revient sur la vitre. Ça sent le poireau. Papa tourne la soupe. Tu as faim, Victorina ? Victorina s'approche de la table. Elle a encore le ventre serré. Le soleil peint est dans le cartable.</t>
+          <t>Victorina connaît le préau, ses crochets, son zinc. Après la pluie, un détail paraît nouveau. Les manteaux jaunes gouttent sur les crochets. Ça sent la laine mouillée, un peu froide. Une goutte tombe de la gouttière de l'école. Le zinc fait un petit chant, tu l'entends ? Oui, papa. Il tombe près des manteaux. Tes cheveux sont prêts, Victorina. Oui, maman. Maman boutonne le manteau jaune. Le tissu est lourd, un peu froid. Le manteau jaune est boutonné ? Oui, maman. Maman glisse un biscuit dans la poche. Le biscuit sent le beurre. Il est pour plus tard. Je peins les manteaux, maintenant ! À l'atelier, près des pots ? Oui, tout de suite ! On y va ? On y va. Au revoir, maman. Au revoir, Victorina. Le préau brille sous les gouttes. Les crochets claquent un peu. En ce moment, Victorina pousse la porte de l'atelier. Ça sent le papier mouillé et l'eau des pots. La nappe de la table est bleue, un peu tâchée. Les pots jaunes sont ouverts. Un pinceau jaune attend près de l'eau. Sur le bois mouillé, un éclat de pinceau brille. Le bois brille, maîtresse. Bonjour les enfants. Bonjour, maîtresse. La maîtresse parle près des pots. Victorina saisit le pinceau jaune. Le bois est lisse, un peu collant. Elle plonge le poil trop vite. L'eau gicle sur la nappe. Le jaune court de travers. Oh. L'éclat de pinceau tremble, puis tient. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Elle essuie la nappe avec un chiffon. Elle reprend le pinceau, plus léger. Une tache jaune ronde tient sur la feuille. C'est le manteau, maîtresse. Oui, Victorina. Victorina va vers le bac. L'eau du bac devient un peu jaune. Elle lave le poil, sans se presser. Près du bac, quelqu'un chuchote. Victorina entend parler d'un secret. Son ventre se serre. Ses joues deviennent chaudes. Je le dis, maintenant ! Elle ouvre la bouche trop vite. Ses mots se cognent à ceux de l'atelier. Personne ne tourne la tête. Oh. Elle referme la bouche. Elle pose le pinceau propre. Elle glisse la feuille dans la poche du manteau. Le soir, la porte de la maison s'ouvre. Ça sent le lait chaud et le pain. Le manteau jaune pend sur la chaise. Te voilà, Victorina. Tes manches sont un peu mouillées. Viens près de la table. Victorina pose le biscuit sur le bois. Elle s'assoit. Le ventre est serré, tout petit. Elle regarde papa. Elle ouvre la bouche.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Denis est à l'école. C'est l'atelier peinture. La maîtresse parle. Denis aime &lt;emphasis level="moderate"&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : on lave les pinceaux. Denis lave son pinceau. Il écoute bien. Plus tard, un camarade chuchote près du bac. Il dit : c'est un secret. Ne le dis pas à la maison. Denis sent un malaise. Son ventre est serré. Le soir, papa prépare la soupe. Ça sent le poireau. Denis vient raconter à la maison. Il dit : papa, j'ai eu un malaise. Un camarade a parlé d'un secret. Maman l'écoute aussi. Papa dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter à papa ou maman.&lt;/prosody&gt;&lt;break time="400ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina connaît le préau, ses crochets, son zinc. Après la pluie, un détail paraît nouveau. Les manteaux jaunes gouttent sur les crochets. Ça sent la laine mouillée, un peu froide. Une goutte tombe de la gouttière de l'école. Le zinc fait un petit chant, tu l'entends ? Oui, papa. Il tombe près des manteaux. Tes cheveux sont prêts, Victorina. Oui, maman. Maman boutonne le manteau jaune. Le tissu est lourd, un peu froid. Le manteau jaune est boutonné ? Oui, maman. Maman glisse un biscuit dans la poche. Le biscuit sent le beurre. Il est pour plus tard. Je peins les manteaux, maintenant ! À l'atelier, près des pots ? Oui, tout de suite ! On y va ? On y va. Au revoir, maman. Au revoir, Victorina. Le préau brille sous les gouttes. Les crochets claquent un peu. En ce moment, Victorina pousse la porte de l'atelier. Ça sent le papier mouillé et l'eau des pots. La nappe de la table est bleue, un peu tâchée. Les pots jaunes sont ouverts. Un pinceau jaune attend près de l'eau. Sur le bois mouillé, un &lt;emphasis level="moderate"&gt;éclat de pinceau&lt;/emphasis&gt; brille. Le bois brille, maîtresse. Bonjour les enfants. Bonjour, maîtresse. La maîtresse parle près des pots. Victorina saisit le pinceau jaune. Le bois est lisse, un peu collant. Elle plonge le poil trop vite. L'eau gicle sur la nappe. Le jaune court de travers. Oh. L'éclat de pinceau tremble, puis tient. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Elle essuie la nappe avec un chiffon. Elle reprend le pinceau, plus léger. Une tache jaune ronde tient sur la feuille. C'est le manteau, maîtresse. Oui, Victorina. Victorina va vers le bac. L'eau du bac devient un peu jaune. Elle lave le poil, sans se presser. Près du bac, quelqu'un chuchote. Victorina entend parler d'un secret. Son ventre se serre. Ses joues deviennent chaudes. Je le dis, maintenant ! Elle ouvre la bouche trop vite. Ses mots se cognent à ceux de l'atelier. Personne ne tourne la tête. Oh. Elle referme la bouche. Elle pose le pinceau propre. Elle glisse la feuille dans la poche du manteau. Le soir, la porte de la maison s'ouvre. Ça sent le lait chaud et le pain. Le manteau jaune pend sur la chaise. Te voilà, Victorina. Tes manches sont un peu mouillées. Viens près de la table. Victorina pose le biscuit sur le bois. Elle s'assoit. Le ventre est serré, tout petit. Elle regarde papa. Elle ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Denis est à l'école. C'est l'atelier peinture. La maîtresse parle. Denis aime &lt;emphasis&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : on lave les pinceaux. Denis lave son pinceau. Il écoute bien. Plus tard, un camarade chuchote près du bac. Il dit : c'est un secret. Ne le dis pas à la maison. Denis sent un malaise. Son ventre est serré. Le soir, papa prépare la soupe. Ça sent le poireau. Denis vient raconter à la maison. Il dit : papa, j'ai eu un malaise. Un camarade a parlé d'un secret. Maman l'écoute aussi. Papa dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter à papa ou maman. [pause]</t>
+          <t>Victorina connaît le préau, ses crochets, son zinc. Après la pluie, un détail paraît nouveau. Les manteaux jaunes gouttent sur les crochets. Ça sent la laine mouillée, un peu froide. Une goutte tombe de la gouttière de l'école. Le zinc fait un petit chant, tu l'entends ? Oui, papa. Il tombe près des manteaux. Tes cheveux sont prêts, Victorina. Oui, maman. Maman boutonne le manteau jaune. Le tissu est lourd, un peu froid. Le manteau jaune est boutonné ? Oui, maman. Maman glisse un biscuit dans la poche. Le biscuit sent le beurre. Il est pour plus tard. Je peins les manteaux, maintenant ! À l'atelier, près des pots ? Oui, tout de suite ! On y va ? On y va. Au revoir, maman. Au revoir, Victorina. Le préau brille sous les gouttes. Les crochets claquent un peu. En ce moment, Victorina pousse la porte de l'atelier. Ça sent le papier mouillé et l'eau des pots. La nappe de la table est bleue, un peu tâchée. Les pots jaunes sont ouverts. Un pinceau jaune attend près de l'eau. Sur le bois mouillé, un &lt;emphasis&gt;éclat de pinceau&lt;/emphasis&gt; brille. Le bois brille, maîtresse. Bonjour les enfants. Bonjour, maîtresse. La maîtresse parle près des pots. Victorina saisit le pinceau jaune. Le bois est lisse, un peu collant. Elle plonge le poil trop vite. L'eau gicle sur la nappe. Le jaune court de travers. Oh. L'éclat de pinceau tremble, puis tient. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Elle essuie la nappe avec un chiffon. Elle reprend le pinceau, plus léger. Une tache jaune ronde tient sur la feuille. C'est le manteau, maîtresse. Oui, Victorina. Victorina va vers le bac. L'eau du bac devient un peu jaune. Elle lave le poil, sans se presser. Près du bac, quelqu'un chuchote. Victorina entend parler d'un secret. Son ventre se serre. Ses joues deviennent chaudes. Je le dis, maintenant ! Elle ouvre la bouche trop vite. Ses mots se cognent à ceux de l'atelier. Personne ne tourne la tête. Oh. Elle referme la bouche. Elle pose le pinceau propre. Elle glisse la feuille dans la poche du manteau. Le soir, la porte de la maison s'ouvre. Ça sent le lait chaud et le pain. Le manteau jaune pend sur la chaise. Te voilà, Victorina. Tes manches sont un peu mouillées. Viens près de la table. Victorina pose le biscuit sur le bois. Elle s'assoit. Le ventre est serré, tout petit. Elle regarde papa. Elle ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>éclat de pinceau</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,67 +1326,96 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_peindre_et_parler_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La casserole frémit sur le feu.
-narrateur|Une buée ronde s'étale sur la vitre.
-narrateur|Ça sent l'orange pelée, un peu vive.
-narrateur|Les gouttes d'huile brillent sur les doigts de maman.
-narrateur|Papa essuie la table avec une éponge jaune.
-narrateur|L'éponge est froide, encore mouillée.
-narrateur|Dehors, le village est gris et calme.
-papa|Victorina, tu vois le rond sur la vitre ?
+          <t>narrateur|Victorina connaît le préau, ses crochets, son zinc.
+narrateur|Après la pluie, un détail paraît nouveau.
+narrateur|Les manteaux jaunes gouttent sur les crochets.
+narrateur|Ça sent la laine mouillée, un peu froide.
+narrateur|Une goutte tombe de la gouttière de l'école.
+papa|Le zinc fait un petit chant, tu l'entends ?
 enfant-f|Oui, papa.
-enfant-f|On dirait un soleil.
-enfant-f|Maman, je veux un vrai soleil, en jaune.
-enfant-f|Pour la fenêtre de la cuisine.
-maman|On pourra le peindre à l'école.
-maman|Tu écoutes la maîtresse, d'accord ?
+enfant-f|Il tombe près des manteaux.
+maman|Tes cheveux sont prêts, Victorina.
 enfant-f|Oui, maman.
-narrateur|Papa glisse un biscuit dans la poche.
+narrateur|Maman boutonne le manteau jaune.
+narrateur|Le tissu est lourd, un peu froid.
+maman|Le manteau jaune est boutonné ?
+enfant-f|Oui, maman.
+narrateur|Maman glisse un biscuit dans la poche.
 narrateur|Le biscuit sent le beurre.
-papa|Il est pour plus tard.
+maman|Il est pour plus tard.
+enfant-f|Je peins les manteaux, maintenant !
+papa|À l'atelier, près des pots ?
+enfant-f|Oui, tout de suite !
+papa|On y va ?
+enfant-f|On y va.
+enfant-f|Au revoir, maman.
+maman|Au revoir, Victorina.
+narrateur|Le préau brille sous les gouttes.
+narrateur|Les crochets claquent un peu.
 narrateur|En ce moment, Victorina pousse la porte de l'atelier.
-narrateur|La table a une nappe bleue, un peu tâchée.
-narrateur|Les pots de peinture sont ouverts.
-narrateur|Ça sent le papier mouillé.
-narrateur|Un pinceau attend près de l'eau.
-maitresse|On écoute d'abord.
-maitresse|Ensuite, on peint un rond.
-maitresse|Puis on lave les pinceaux.
-narrateur|Victorina aime écouter.
-narrateur|Elle prend le pinceau.
+narrateur|Ça sent le papier mouillé et l'eau des pots.
+narrateur|La nappe de la table est bleue, un peu tâchée.
+narrateur|Les pots jaunes sont ouverts.
+narrateur|Un pinceau jaune attend près de l'eau.
+narrateur|Sur le bois mouillé, un éclat de pinceau brille.
+enfant-f|Le bois brille, maîtresse.
+maitresse|Bonjour les enfants.
+enfant-f|Bonjour, maîtresse.
+narrateur|La maîtresse parle près des pots.
+narrateur|Victorina saisit le pinceau jaune.
 narrateur|Le bois est lisse, un peu collant.
-narrateur|Elle plonge le poil dans le jaune.
-narrateur|Le jaune est épais.
-enfant-f|C'est mon soleil, maîtresse.
+narrateur|Elle plonge le poil trop vite.
+narrateur|L'eau gicle sur la nappe.
+narrateur|Le jaune court de travers.
+enfant-f|Oh.
+narrateur|L'éclat de pinceau tremble, puis tient.
+narrateur|Le sourire de Victorina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Ça ne veut pas.
+narrateur|Ses épaules tombent un peu.
+narrateur|Elle essuie la nappe avec un chiffon.
+narrateur|Elle reprend le pinceau, plus léger.
+narrateur|Une tache jaune ronde tient sur la feuille.
+enfant-f|C'est le manteau, maîtresse.
 maitresse|Oui, Victorina.
-maitresse|Tu as bien écouté.
-maitresse|Maintenant, on lave les pinceaux.
 narrateur|Victorina va vers le bac.
-narrateur|L'eau devient un peu jaune.
-narrateur|Elle lave le poil, tout doucement.
-narrateur|Le soleil reste sur la feuille, encore humide.
-narrateur|Près du bac, quelqu'un parle tout bas.
+narrateur|L'eau du bac devient un peu jaune.
+narrateur|Elle lave le poil, sans se presser.
+narrateur|Près du bac, quelqu'un chuchote.
 narrateur|Victorina entend parler d'un secret.
 narrateur|Son ventre se serre.
 narrateur|Ses joues deviennent chaudes.
+enfant-f|Je le dis, maintenant !
+narrateur|Elle ouvre la bouche trop vite.
+narrateur|Ses mots se cognent à ceux de l'atelier.
+narrateur|Personne ne tourne la tête.
+enfant-f|Oh.
+narrateur|Elle referme la bouche.
 narrateur|Elle pose le pinceau propre.
-enfant-f|Je raconterai à la maison.
-narrateur|Le soir, la casserole frémit encore.
-narrateur|La buée revient sur la vitre.
-narrateur|Ça sent le poireau.
-narrateur|Papa tourne la soupe.
-papa|Tu as faim, Victorina ?
-narrateur|Victorina s'approche de la table.
-narrateur|Elle a encore le ventre serré.
-narrateur|Le soleil peint est dans le cartable.</t>
+narrateur|Elle glisse la feuille dans la poche du manteau.
+narrateur|Le soir, la porte de la maison s'ouvre.
+narrateur|Ça sent le lait chaud et le pain.
+narrateur|Le manteau jaune pend sur la chaise.
+papa|Te voilà, Victorina.
+papa|Tes manches sont un peu mouillées.
+maman|Viens près de la table.
+narrateur|Victorina pose le biscuit sur le bois.
+narrateur|Elle s'assoit.
+narrateur|Le ventre est serré, tout petit.
+narrateur|Elle regarde papa.
+narrateur|Elle ouvre la bouche.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>casserole,eau</t>
+          <t>pluie,eau</t>
         </is>
       </c>
     </row>
@@ -1418,12 +1447,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Denis a un malaise. Que fait-il ?&lt;/prosody&gt;&lt;break time="250ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorina a un &lt;emphasis level="moderate"&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Denis a un malaise. Que fait-il ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorina a un &lt;emphasis&gt;malaise&lt;/emphasis&gt;. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1486,18 +1515,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1512,34 +1541,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>malaise</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1548,23 +1581,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_raconte_quand_le_ventre_serre; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1597,17 +1630,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Papa, j'ai eu un malaise. Quelqu'un a parlé d'un secret. Maman pose la louche. Tu as bien fait de raconter. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter. À papa ou à maman. Victorina respire. Son ventre se desserre, tout doucement. J'ai peint un soleil. Il est dans le cartable. On le sort ? Oui. Papa ouvre le cartable. La feuille est un peu gondolée. Le jaune brille encore. Il est rond, comme la buée. Tu as écouté, puis tu as peint.</t>
+          <t>Victorina ouvre la bouche trop vite. Papa, quelqu'un a parlé. Papa n'a pas fini sa phrase. Le lait est chaud, Victorina. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Papa se baisse à sa hauteur. Victorina refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la cuisine, un instant. Tes manches sèchent sur la chaise ? Papa pose son bol. Le lait fume un peu. Maman n'a pas fini non plus. Victorina attend que le silence arrive. Sur la feuille, un éclat de pinceau brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Quelqu'un a parlé d'un secret. Mon ventre s'est serré, à l'atelier. Merci, Victorina. Papa a entendu toute la phrase. Tu as fini ton lait ? Presque, maman. Le ventre de Victorina se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Denis a écouté la maîtresse. Il a raconté son malaise à la maison. Papa et maman sont là.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina ouvre la bouche trop vite. Papa, quelqu'un a parlé. Papa n'a pas fini sa phrase. Le lait est chaud, Victorina. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Papa se baisse à sa hauteur. Victorina refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la cuisine, un instant. Tes manches sèchent sur la chaise ? Papa pose son bol. Le lait fume un peu. Maman n'a pas fini non plus. Victorina attend que le &lt;emphasis level="moderate"&gt;silence&lt;/emphasis&gt; arrive. Sur la feuille, un éclat de pinceau brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Quelqu'un a parlé d'un secret. Mon ventre s'est serré, à l'atelier. Merci, Victorina. Papa a entendu toute la phrase. Tu as fini ton lait ? Presque, maman. Le ventre de Victorina se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Denis a écouté la maîtresse. Il a raconté son malaise à la maison. Papa et maman sont là. [pause]</t>
+          <t>Victorina ouvre la bouche trop vite. Papa, quelqu'un a parlé. Papa n'a pas fini sa phrase. Le lait est chaud, Victorina. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Papa se baisse à sa hauteur. Victorina refuse de foncer. Elle referme la bouche. Elle pose les mains à plat. Elle écoute la cuisine, un instant. Tes manches sèchent sur la chaise ? Papa pose son bol. Le lait fume un peu. Maman n'a pas fini non plus. Victorina attend que le &lt;emphasis&gt;silence&lt;/emphasis&gt; arrive. Sur la feuille, un éclat de pinceau brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Quelqu'un a parlé d'un secret. Mon ventre s'est serré, à l'atelier. Merci, Victorina. Papa a entendu toute la phrase. Tu as fini ton lait ? Presque, maman. Le ventre de Victorina se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1654,7 +1687,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1662,10 +1695,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1686,28 +1719,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>silence</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1716,10 +1753,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1732,29 +1769,39 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-f|Papa, j'ai eu un malaise.
+          <t>narrateur|Victorina ouvre la bouche trop vite.
+enfant-f|Papa, quelqu'un a parlé.
+narrateur|Papa n'a pas fini sa phrase.
+papa|Le lait est chaud, Victorina.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Papa se baisse à sa hauteur.
+narrateur|Victorina refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Elle pose les mains à plat.
+narrateur|Elle écoute la cuisine, un instant.
+papa|Tes manches sèchent sur la chaise ?
+narrateur|Papa pose son bol.
+maman|Le lait fume un peu.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Victorina attend que le silence arrive.
+narrateur|Sur la feuille, un éclat de pinceau brille.
+enfant-f|Il est là.
+enfant-f|Je peux te dire quelque chose ?
+maman|Oui, nous t'écoutons.
 enfant-f|Quelqu'un a parlé d'un secret.
-narrateur|Maman pose la louche.
-maman|Tu as bien fait de raconter.
-maman|On aime écouter la maîtresse.
-papa|Si tu as un malaise, tu viens raconter.
-papa|À papa ou à maman.
-narrateur|Victorina respire.
-narrateur|Son ventre se desserre, tout doucement.
-enfant-f|J'ai peint un soleil.
-enfant-f|Il est dans le cartable.
-maman|On le sort ?
-enfant-f|Oui.
-narrateur|Papa ouvre le cartable.
-narrateur|La feuille est un peu gondolée.
-narrateur|Le jaune brille encore.
-papa|Il est rond, comme la buée.
-maman|Tu as écouté, puis tu as peint.</t>
+enfant-f|Mon ventre s'est serré, à l'atelier.
+papa|Merci, Victorina.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu as fini ton lait ?
+enfant-f|Presque, maman.
+narrateur|Le ventre de Victorina se desserre.</t>
         </is>
       </c>
     </row>
@@ -1781,17 +1828,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Papa tient la feuille contre la vitre. La buée fait un halo autour du jaune. Le soleil est à sa place. Tu veux un peu d'eau ? Oui, maman. Victorina boit une gorgée. L'eau est fraîche. Je te tiens la main ? Oui, papa. Sa main est chaude. Le biscuit est encore dans ta poche. Tu le manges après la soupe ? Oui. La casserole frémit plus bas. La cuisine est calme.</t>
+          <t>Victorina sort la feuille de la poche. Le papier est un peu gondolé. Le pinceau de la boîte est là. Maman pose un verre d'eau sur le bois. Un petit pinceau attend dans le verre. Je peins les manteaux. Tu leur fais une place sur la feuille ? Oui. Ici, au milieu. Victorina veut tracer tout de suite. Elle appuie trop fort. Le jaune court de travers. Oh. Elle s'arrête. Ses mains se ferment, puis s'ouvrent. Elle refuse de foncer. Elle écoute la pluie, un instant. Elle reprend le pinceau, plus léger. Une ligne jaune descend, comme un manteau. On voit presque les crochets. Victorina ajoute une petite poche ronde. Et le biscuit, dedans ? Un biscuit, oui. Elle souffle sur la feuille. Fffff. La pluie ralentit derrière la vitre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Denis boit un verre d'eau. Papa lui tient la &lt;emphasis level="moderate"&gt;main&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina sort la feuille de la poche. Le papier est un peu gondolé. Le &lt;emphasis level="moderate"&gt;pinceau&lt;/emphasis&gt; de la boîte est là. Maman pose un verre d'eau sur le bois. Un petit pinceau attend dans le verre. Je peins les manteaux. Tu leur fais une place sur la feuille ? Oui. Ici, au milieu. Victorina veut tracer tout de suite. Elle appuie trop fort. Le jaune court de travers. Oh. Elle s'arrête. Ses mains se ferment, puis s'ouvrent. Elle refuse de foncer. Elle écoute la pluie, un instant. Elle reprend le pinceau, plus léger. Une ligne jaune descend, comme un manteau. On voit presque les crochets. Victorina ajoute une petite poche ronde. Et le biscuit, dedans ? Un biscuit, oui. Elle souffle sur la feuille. Fffff. La pluie ralentit derrière la vitre.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Denis boit un verre d'eau. Papa lui tient la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Victorina sort la feuille de la poche. Le papier est un peu gondolé. Le &lt;emphasis&gt;pinceau&lt;/emphasis&gt; de la boîte est là. Maman pose un verre d'eau sur le bois. Un petit pinceau attend dans le verre. Je peins les manteaux. Tu leur fais une place sur la feuille ? Oui. Ici, au milieu. Victorina veut tracer tout de suite. Elle appuie trop fort. Le jaune court de travers. Oh. Elle s'arrête. Ses mains se ferment, puis s'ouvrent. Elle refuse de foncer. Elle écoute la pluie, un instant. Elle reprend le pinceau, plus léger. Une ligne jaune descend, comme un manteau. On voit presque les crochets. Victorina ajoute une petite poche ronde. Et le biscuit, dedans ? Un biscuit, oui. Elle souffle sur la feuille. Fffff. La pluie ralentit derrière la vitre. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1838,7 +1885,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1846,10 +1893,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1872,30 +1919,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>pinceau</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1904,10 +1951,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1918,24 +1965,39 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sur_la_feuille; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Papa tient la feuille contre la vitre.
-narrateur|La buée fait un halo autour du jaune.
-enfant-f|Le soleil est à sa place.
-maman|Tu veux un peu d'eau ?
-enfant-f|Oui, maman.
-narrateur|Victorina boit une gorgée.
-narrateur|L'eau est fraîche.
-papa|Je te tiens la main ?
-enfant-f|Oui, papa.
-narrateur|Sa main est chaude.
-maman|Le biscuit est encore dans ta poche.
-maman|Tu le manges après la soupe ?
+          <t>narrateur|Victorina sort la feuille de la poche.
+narrateur|Le papier est un peu gondolé.
+maman|Le pinceau de la boîte est là.
+narrateur|Maman pose un verre d'eau sur le bois.
+narrateur|Un petit pinceau attend dans le verre.
+enfant-f|Je peins les manteaux.
+papa|Tu leur fais une place sur la feuille ?
 enfant-f|Oui.
-narrateur|La casserole frémit plus bas.
-narrateur|La cuisine est calme.</t>
+enfant-f|Ici, au milieu.
+narrateur|Victorina veut tracer tout de suite.
+narrateur|Elle appuie trop fort.
+narrateur|Le jaune court de travers.
+enfant-f|Oh.
+narrateur|Elle s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Elle refuse de foncer.
+narrateur|Elle écoute la pluie, un instant.
+narrateur|Elle reprend le pinceau, plus léger.
+narrateur|Une ligne jaune descend, comme un manteau.
+maman|On voit presque les crochets.
+narrateur|Victorina ajoute une petite poche ronde.
+papa|Et le biscuit, dedans ?
+enfant-f|Un biscuit, oui.
+narrateur|Elle souffle sur la feuille.
+enfant-f|Fffff.
+narrateur|La pluie ralentit derrière la vitre.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1967,17 +2029,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Mon soleil est sur la vitre. J'ai écouté. Puis j'ai raconté. On t'a écoutée aussi. Bravo, Victorina.</t>
+          <t>Le manteau jaune sèche sur la chaise. La feuille jaune reste sur la table. Comme à l'atelier, papa ! Tu le vois, toi ? Oui, sur le jaune. On est bien, ici. Le lait fume un peu, près de la fenêtre. Victorina glisse le pinceau sans se presser. Le bois repose contre la feuille. Il brille, maman. Tu le vois sur le papier ? Oui, sur le jaune. La pluie reste dans l'air. L'éclat de pinceau tient sur le jaune.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Mon soleil est sur la vitre. J'ai écouté. Puis j'ai raconté. On t'a écoutée aussi. Bravo, Victorina.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le manteau jaune sèche sur la chaise. La feuille jaune reste sur la table. Comme à l'atelier, papa ! Tu le vois, toi ? Oui, sur le jaune. On est bien, ici. Le lait fume un peu, près de la fenêtre. Victorina glisse le pinceau sans se presser. Le bois repose contre la feuille. Il brille, maman. Tu le vois sur le papier ? Oui, sur le jaune. La pluie reste dans l'air. L'&lt;emphasis level="moderate"&gt;éclat de pinceau&lt;/emphasis&gt; tient sur le jaune.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le manteau jaune sèche sur la chaise. La feuille jaune reste sur la table. Comme à l'atelier, papa ! Tu le vois, toi ? Oui, sur le jaune. On est bien, ici. Le lait fume un peu, près de la fenêtre. Victorina glisse le pinceau sans se presser. Le bois repose contre la feuille. Il brille, maman. Tu le vois sur le papier ? Oui, sur le jaune. La pluie reste dans l'air. L'&lt;emphasis&gt;éclat de pinceau&lt;/emphasis&gt; tient sur le jaune.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2024,18 +2086,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2044,12 +2106,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2058,17 +2120,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pinceau</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2077,11 +2143,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2090,28 +2156,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_jaune; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|Mon soleil est sur la vitre.
-enfant-f|J'ai écouté.
-enfant-f|Puis j'ai raconté.
-maman|On t'a écoutée aussi.
-papa|Bravo, Victorina.</t>
+          <t>narrateur|Le manteau jaune sèche sur la chaise.
+narrateur|La feuille jaune reste sur la table.
+enfant-f|Comme à l'atelier, papa !
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur le jaune.
+maman|On est bien, ici.
+narrateur|Le lait fume un peu, près de la fenêtre.
+narrateur|Victorina glisse le pinceau sans se presser.
+narrateur|Le bois repose contre la feuille.
+enfant-f|Il brille, maman.
+maman|Tu le vois sur le papier ?
+enfant-f|Oui, sur le jaune.
+narrateur|La pluie reste dans l'air.
+narrateur|L'éclat de pinceau tient sur le jaune.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pluie</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2217,6 +2301,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>